<commit_message>
Tablas_Stock archivo v2 - Jun-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_06.xlsx
+++ b/Tablas/Tablas_Stock_2026_06.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 70% (+6pp vs mayo). Muestra en maduracion: tasa de respuesta 3.5% (149 respuestas), las 7 areas por debajo del 5%. Dato publicado con reserva por representatividad.</t>
+          <t>Satisfaccion global 70% (+6pp vs mayo). (*) Muestra escasa: en junio se registraron inconvenientes tecnicos en la toma de encuestas, sumado a la maduracion natural de respuestas. Tasa 3.5% (149 resp.), 7 areas &lt;5%. Dato con reserva.</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Tasa de respuesta de encuesta 3.5% en Jun-2026 (149 respuestas sobre 4309 incidentes); las 7 areas del monitor quedan por debajo del 5%. La baja responde a la maduracion de la encuesta (las respuestas de Jun-2026 aun no se acumularon al corte), no a una caida de satisfaccion. La satisfaccion por area se publica con la marca '(muestra insuficiente)'.</t>
+          <t>Tasa de respuesta de encuesta 3.5% en Jun-2026 (149 respuestas sobre 4309 incidentes); las 7 areas del monitor quedan por debajo del 5%. Dos causas: inconvenientes tecnicos en la toma de encuestas durante Jun-2026 y la maduracion natural de las respuestas (las cargadas en Jun-2026 aun no se acumularon al corte). No refleja caida de satisfaccion. La satisfaccion por area se publica con la marca '(muestra insuficiente)'.</t>
         </is>
       </c>
     </row>

</xml_diff>